<commit_message>
Add simple trapezoid section figure for y=0.25/0.30/0.35
Embed a plain schematic and x/Tw table in the ditch workbook for
office presentation.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/Fosse_trapezoidal_largeur_fond_x.xlsx
+++ b/engineering/drainage-design/Fosse_trapezoidal_largeur_fond_x.xlsx
@@ -8,11 +8,12 @@
   </bookViews>
   <sheets>
     <sheet name="Resultats" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Guide" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Inputs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Exemple_pas_a_pas" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Comparaison_n" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Solveur_optionnel" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Figure_section" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Guide" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Inputs" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Exemple_pas_a_pas" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Comparaison_n" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Solveur_optionnel" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,11 +23,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="0.0000"/>
-    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,6 +52,20 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
   <fills count="7">
@@ -112,11 +127,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -124,10 +139,10 @@
     <xf numFmtId="2" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -138,16 +153,35 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -239,6 +273,36 @@
     </comment>
   </commentList>
 </comments>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6572250" cy="3000375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -570,7 +634,7 @@
           <t>Q=</t>
         </is>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="23">
         <f>Inputs!B4</f>
         <v/>
       </c>
@@ -579,7 +643,7 @@
           <t>S=</t>
         </is>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="24">
         <f>Inputs!B5</f>
         <v/>
       </c>
@@ -588,7 +652,7 @@
           <t>n=</t>
         </is>
       </c>
-      <c r="G3" s="2">
+      <c r="G3" s="23">
         <f>Inputs!B6</f>
         <v/>
       </c>
@@ -667,30 +731,30 @@
       <c r="A6" s="6" t="n">
         <v>0.2</v>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="25" t="n">
         <v>11.917</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="26">
         <f>($B6+$I$3*$A6)*$A6</f>
         <v/>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="26">
         <f>$B6+2*$A6*SQRT(1+$I$3^2)</f>
         <v/>
       </c>
-      <c r="E6" s="8">
+      <c r="E6" s="26">
         <f>C6/D6</f>
         <v/>
       </c>
-      <c r="F6" s="8">
+      <c r="F6" s="26">
         <f>$B6+2*$I$3*$A6</f>
         <v/>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="26">
         <f>(1/$G$3)*C6*E6^(2/3)*SQRT($E$3)</f>
         <v/>
       </c>
-      <c r="H6" s="8">
+      <c r="H6" s="26">
         <f>G6/C6</f>
         <v/>
       </c>
@@ -707,30 +771,30 @@
       <c r="A7" s="6" t="n">
         <v>0.25</v>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="25" t="n">
         <v>8.161</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="26">
         <f>($B7+$I$3*$A7)*$A7</f>
         <v/>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="26">
         <f>$B7+2*$A7*SQRT(1+$I$3^2)</f>
         <v/>
       </c>
-      <c r="E7" s="8">
+      <c r="E7" s="26">
         <f>C7/D7</f>
         <v/>
       </c>
-      <c r="F7" s="8">
+      <c r="F7" s="26">
         <f>$B7+2*$I$3*$A7</f>
         <v/>
       </c>
-      <c r="G7" s="8">
+      <c r="G7" s="26">
         <f>(1/$G$3)*C7*E7^(2/3)*SQRT($E$3)</f>
         <v/>
       </c>
-      <c r="H7" s="8">
+      <c r="H7" s="26">
         <f>G7/C7</f>
         <v/>
       </c>
@@ -747,30 +811,30 @@
       <c r="A8" s="6" t="n">
         <v>0.3</v>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="25" t="n">
         <v>5.956</v>
       </c>
-      <c r="C8" s="8">
+      <c r="C8" s="26">
         <f>($B8+$I$3*$A8)*$A8</f>
         <v/>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="26">
         <f>$B8+2*$A8*SQRT(1+$I$3^2)</f>
         <v/>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="26">
         <f>C8/D8</f>
         <v/>
       </c>
-      <c r="F8" s="8">
+      <c r="F8" s="26">
         <f>$B8+2*$I$3*$A8</f>
         <v/>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="26">
         <f>(1/$G$3)*C8*E8^(2/3)*SQRT($E$3)</f>
         <v/>
       </c>
-      <c r="H8" s="8">
+      <c r="H8" s="26">
         <f>G8/C8</f>
         <v/>
       </c>
@@ -787,30 +851,30 @@
       <c r="A9" s="6" t="n">
         <v>0.35</v>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="25" t="n">
         <v>4.529</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="26">
         <f>($B9+$I$3*$A9)*$A9</f>
         <v/>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="26">
         <f>$B9+2*$A9*SQRT(1+$I$3^2)</f>
         <v/>
       </c>
-      <c r="E9" s="8">
+      <c r="E9" s="26">
         <f>C9/D9</f>
         <v/>
       </c>
-      <c r="F9" s="8">
+      <c r="F9" s="26">
         <f>$B9+2*$I$3*$A9</f>
         <v/>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="26">
         <f>(1/$G$3)*C9*E9^(2/3)*SQRT($E$3)</f>
         <v/>
       </c>
-      <c r="H9" s="8">
+      <c r="H9" s="26">
         <f>G9/C9</f>
         <v/>
       </c>
@@ -827,30 +891,30 @@
       <c r="A10" s="6" t="n">
         <v>0.4</v>
       </c>
-      <c r="B10" s="7" t="n">
+      <c r="B10" s="25" t="n">
         <v>3.534</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="26">
         <f>($B10+$I$3*$A10)*$A10</f>
         <v/>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="26">
         <f>$B10+2*$A10*SQRT(1+$I$3^2)</f>
         <v/>
       </c>
-      <c r="E10" s="8">
+      <c r="E10" s="26">
         <f>C10/D10</f>
         <v/>
       </c>
-      <c r="F10" s="8">
+      <c r="F10" s="26">
         <f>$B10+2*$I$3*$A10</f>
         <v/>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="26">
         <f>(1/$G$3)*C10*E10^(2/3)*SQRT($E$3)</f>
         <v/>
       </c>
-      <c r="H10" s="8">
+      <c r="H10" s="26">
         <f>G10/C10</f>
         <v/>
       </c>
@@ -867,30 +931,30 @@
       <c r="A11" s="6" t="n">
         <v>0.5</v>
       </c>
-      <c r="B11" s="7" t="n">
+      <c r="B11" s="25" t="n">
         <v>2.233</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="26">
         <f>($B11+$I$3*$A11)*$A11</f>
         <v/>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="26">
         <f>$B11+2*$A11*SQRT(1+$I$3^2)</f>
         <v/>
       </c>
-      <c r="E11" s="8">
+      <c r="E11" s="26">
         <f>C11/D11</f>
         <v/>
       </c>
-      <c r="F11" s="8">
+      <c r="F11" s="26">
         <f>$B11+2*$I$3*$A11</f>
         <v/>
       </c>
-      <c r="G11" s="8">
+      <c r="G11" s="26">
         <f>(1/$G$3)*C11*E11^(2/3)*SQRT($E$3)</f>
         <v/>
       </c>
-      <c r="H11" s="8">
+      <c r="H11" s="26">
         <f>G11/C11</f>
         <v/>
       </c>
@@ -907,30 +971,30 @@
       <c r="A12" s="6" t="n">
         <v>0.6</v>
       </c>
-      <c r="B12" s="7" t="n">
+      <c r="B12" s="25" t="n">
         <v>1.398</v>
       </c>
-      <c r="C12" s="8">
+      <c r="C12" s="26">
         <f>($B12+$I$3*$A12)*$A12</f>
         <v/>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="26">
         <f>$B12+2*$A12*SQRT(1+$I$3^2)</f>
         <v/>
       </c>
-      <c r="E12" s="8">
+      <c r="E12" s="26">
         <f>C12/D12</f>
         <v/>
       </c>
-      <c r="F12" s="8">
+      <c r="F12" s="26">
         <f>$B12+2*$I$3*$A12</f>
         <v/>
       </c>
-      <c r="G12" s="8">
+      <c r="G12" s="26">
         <f>(1/$G$3)*C12*E12^(2/3)*SQRT($E$3)</f>
         <v/>
       </c>
-      <c r="H12" s="8">
+      <c r="H12" s="26">
         <f>G12/C12</f>
         <v/>
       </c>
@@ -947,30 +1011,30 @@
       <c r="A13" s="6" t="n">
         <v>0.7</v>
       </c>
-      <c r="B13" s="7" t="n">
+      <c r="B13" s="25" t="n">
         <v>0.792</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="26">
         <f>($B13+$I$3*$A13)*$A13</f>
         <v/>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="26">
         <f>$B13+2*$A13*SQRT(1+$I$3^2)</f>
         <v/>
       </c>
-      <c r="E13" s="8">
+      <c r="E13" s="26">
         <f>C13/D13</f>
         <v/>
       </c>
-      <c r="F13" s="8">
+      <c r="F13" s="26">
         <f>$B13+2*$I$3*$A13</f>
         <v/>
       </c>
-      <c r="G13" s="8">
+      <c r="G13" s="26">
         <f>(1/$G$3)*C13*E13^(2/3)*SQRT($E$3)</f>
         <v/>
       </c>
-      <c r="H13" s="8">
+      <c r="H13" s="26">
         <f>G13/C13</f>
         <v/>
       </c>
@@ -987,30 +1051,30 @@
       <c r="A14" s="6" t="n">
         <v>0.76</v>
       </c>
-      <c r="B14" s="7" t="n">
+      <c r="B14" s="25" t="n">
         <v>0.492</v>
       </c>
-      <c r="C14" s="8">
+      <c r="C14" s="26">
         <f>($B14+$I$3*$A14)*$A14</f>
         <v/>
       </c>
-      <c r="D14" s="8">
+      <c r="D14" s="26">
         <f>$B14+2*$A14*SQRT(1+$I$3^2)</f>
         <v/>
       </c>
-      <c r="E14" s="8">
+      <c r="E14" s="26">
         <f>C14/D14</f>
         <v/>
       </c>
-      <c r="F14" s="8">
+      <c r="F14" s="26">
         <f>$B14+2*$I$3*$A14</f>
         <v/>
       </c>
-      <c r="G14" s="8">
+      <c r="G14" s="26">
         <f>(1/$G$3)*C14*E14^(2/3)*SQRT($E$3)</f>
         <v/>
       </c>
-      <c r="H14" s="8">
+      <c r="H14" s="26">
         <f>G14/C14</f>
         <v/>
       </c>
@@ -1027,30 +1091,30 @@
       <c r="A15" s="6" t="n">
         <v>0.8</v>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="25" t="n">
         <v>0.311</v>
       </c>
-      <c r="C15" s="8">
+      <c r="C15" s="26">
         <f>($B15+$I$3*$A15)*$A15</f>
         <v/>
       </c>
-      <c r="D15" s="8">
+      <c r="D15" s="26">
         <f>$B15+2*$A15*SQRT(1+$I$3^2)</f>
         <v/>
       </c>
-      <c r="E15" s="8">
+      <c r="E15" s="26">
         <f>C15/D15</f>
         <v/>
       </c>
-      <c r="F15" s="8">
+      <c r="F15" s="26">
         <f>$B15+2*$I$3*$A15</f>
         <v/>
       </c>
-      <c r="G15" s="8">
+      <c r="G15" s="26">
         <f>(1/$G$3)*C15*E15^(2/3)*SQRT($E$3)</f>
         <v/>
       </c>
-      <c r="H15" s="8">
+      <c r="H15" s="26">
         <f>G15/C15</f>
         <v/>
       </c>
@@ -1067,30 +1131,30 @@
       <c r="A16" s="6" t="n">
         <v>0.9</v>
       </c>
-      <c r="B16" s="7" t="n">
+      <c r="B16" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="C16" s="8">
+      <c r="C16" s="26">
         <f>($B16+$I$3*$A16)*$A16</f>
         <v/>
       </c>
-      <c r="D16" s="8">
+      <c r="D16" s="26">
         <f>$B16+2*$A16*SQRT(1+$I$3^2)</f>
         <v/>
       </c>
-      <c r="E16" s="8">
+      <c r="E16" s="26">
         <f>C16/D16</f>
         <v/>
       </c>
-      <c r="F16" s="8">
+      <c r="F16" s="26">
         <f>$B16+2*$I$3*$A16</f>
         <v/>
       </c>
-      <c r="G16" s="8">
+      <c r="G16" s="26">
         <f>(1/$G$3)*C16*E16^(2/3)*SQRT($E$3)</f>
         <v/>
       </c>
-      <c r="H16" s="8">
+      <c r="H16" s="26">
         <f>G16/C16</f>
         <v/>
       </c>
@@ -1107,30 +1171,30 @@
       <c r="A17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B17" s="7" t="n">
+      <c r="B17" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="C17" s="8">
+      <c r="C17" s="26">
         <f>($B17+$I$3*$A17)*$A17</f>
         <v/>
       </c>
-      <c r="D17" s="8">
+      <c r="D17" s="26">
         <f>$B17+2*$A17*SQRT(1+$I$3^2)</f>
         <v/>
       </c>
-      <c r="E17" s="8">
+      <c r="E17" s="26">
         <f>C17/D17</f>
         <v/>
       </c>
-      <c r="F17" s="8">
+      <c r="F17" s="26">
         <f>$B17+2*$I$3*$A17</f>
         <v/>
       </c>
-      <c r="G17" s="8">
+      <c r="G17" s="26">
         <f>(1/$G$3)*C17*E17^(2/3)*SQRT($E$3)</f>
         <v/>
       </c>
-      <c r="H17" s="8">
+      <c r="H17" s="26">
         <f>G17/C17</f>
         <v/>
       </c>
@@ -1196,31 +1260,31 @@
       <c r="A22" s="12" t="n">
         <v>0.2</v>
       </c>
-      <c r="B22" s="13">
+      <c r="B22" s="27">
         <f>IFERROR(INDEX(B$6:B$17,MATCH(A22,$A$6:$A$17,0)),"")</f>
         <v/>
       </c>
-      <c r="C22" s="13">
+      <c r="C22" s="27">
         <f>IFERROR(INDEX(C$6:C$17,MATCH(A22,$A$6:$A$17,0)),"")</f>
         <v/>
       </c>
-      <c r="D22" s="13">
+      <c r="D22" s="27">
         <f>IFERROR(INDEX(D$6:D$17,MATCH(A22,$A$6:$A$17,0)),"")</f>
         <v/>
       </c>
-      <c r="E22" s="13">
+      <c r="E22" s="27">
         <f>IFERROR(INDEX(E$6:E$17,MATCH(A22,$A$6:$A$17,0)),"")</f>
         <v/>
       </c>
-      <c r="F22" s="13">
+      <c r="F22" s="27">
         <f>IFERROR(INDEX(F$6:F$17,MATCH(A22,$A$6:$A$17,0)),"")</f>
         <v/>
       </c>
-      <c r="G22" s="13">
+      <c r="G22" s="27">
         <f>IFERROR(INDEX(G$6:G$17,MATCH(A22,$A$6:$A$17,0)),"")</f>
         <v/>
       </c>
-      <c r="H22" s="13">
+      <c r="H22" s="27">
         <f>IFERROR(INDEX(H$6:H$17,MATCH(A22,$A$6:$A$17,0)),"")</f>
         <v/>
       </c>
@@ -1229,31 +1293,31 @@
       <c r="A23" s="12" t="n">
         <v>0.3</v>
       </c>
-      <c r="B23" s="13">
+      <c r="B23" s="27">
         <f>IFERROR(INDEX(B$6:B$17,MATCH(A23,$A$6:$A$17,0)),"")</f>
         <v/>
       </c>
-      <c r="C23" s="13">
+      <c r="C23" s="27">
         <f>IFERROR(INDEX(C$6:C$17,MATCH(A23,$A$6:$A$17,0)),"")</f>
         <v/>
       </c>
-      <c r="D23" s="13">
+      <c r="D23" s="27">
         <f>IFERROR(INDEX(D$6:D$17,MATCH(A23,$A$6:$A$17,0)),"")</f>
         <v/>
       </c>
-      <c r="E23" s="13">
+      <c r="E23" s="27">
         <f>IFERROR(INDEX(E$6:E$17,MATCH(A23,$A$6:$A$17,0)),"")</f>
         <v/>
       </c>
-      <c r="F23" s="13">
+      <c r="F23" s="27">
         <f>IFERROR(INDEX(F$6:F$17,MATCH(A23,$A$6:$A$17,0)),"")</f>
         <v/>
       </c>
-      <c r="G23" s="13">
+      <c r="G23" s="27">
         <f>IFERROR(INDEX(G$6:G$17,MATCH(A23,$A$6:$A$17,0)),"")</f>
         <v/>
       </c>
-      <c r="H23" s="13">
+      <c r="H23" s="27">
         <f>IFERROR(INDEX(H$6:H$17,MATCH(A23,$A$6:$A$17,0)),"")</f>
         <v/>
       </c>
@@ -1262,31 +1326,31 @@
       <c r="A24" s="12" t="n">
         <v>0.4</v>
       </c>
-      <c r="B24" s="13">
+      <c r="B24" s="27">
         <f>IFERROR(INDEX(B$6:B$17,MATCH(A24,$A$6:$A$17,0)),"")</f>
         <v/>
       </c>
-      <c r="C24" s="13">
+      <c r="C24" s="27">
         <f>IFERROR(INDEX(C$6:C$17,MATCH(A24,$A$6:$A$17,0)),"")</f>
         <v/>
       </c>
-      <c r="D24" s="13">
+      <c r="D24" s="27">
         <f>IFERROR(INDEX(D$6:D$17,MATCH(A24,$A$6:$A$17,0)),"")</f>
         <v/>
       </c>
-      <c r="E24" s="13">
+      <c r="E24" s="27">
         <f>IFERROR(INDEX(E$6:E$17,MATCH(A24,$A$6:$A$17,0)),"")</f>
         <v/>
       </c>
-      <c r="F24" s="13">
+      <c r="F24" s="27">
         <f>IFERROR(INDEX(F$6:F$17,MATCH(A24,$A$6:$A$17,0)),"")</f>
         <v/>
       </c>
-      <c r="G24" s="13">
+      <c r="G24" s="27">
         <f>IFERROR(INDEX(G$6:G$17,MATCH(A24,$A$6:$A$17,0)),"")</f>
         <v/>
       </c>
-      <c r="H24" s="13">
+      <c r="H24" s="27">
         <f>IFERROR(INDEX(H$6:H$17,MATCH(A24,$A$6:$A$17,0)),"")</f>
         <v/>
       </c>
@@ -1320,6 +1384,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>Figure — section trapezoïdale et x pour y = 0.25 / 0.30 / 0.35 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Q = 3.598 m3/s ; S = 0.0173 ; n = 0.030 ; talus 2H:1V</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Schema simple pour presentation. Tw = largeur au miroir = x + 4y.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="29" t="inlineStr">
+        <is>
+          <t>Tableau (memes valeurs que la figure)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="30" t="inlineStr">
+        <is>
+          <t>y (m)</t>
+        </is>
+      </c>
+      <c r="B21" s="30" t="inlineStr">
+        <is>
+          <t>x (m)</t>
+        </is>
+      </c>
+      <c r="C21" s="30" t="inlineStr">
+        <is>
+          <t>Tw (m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="18" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="B22" s="31" t="n">
+        <v>8.16</v>
+      </c>
+      <c r="C22" s="31" t="n">
+        <v>9.16</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="18" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="B23" s="31" t="n">
+        <v>5.96</v>
+      </c>
+      <c r="C23" s="31" t="n">
+        <v>7.16</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="B24" s="31" t="n">
+        <v>4.53</v>
+      </c>
+      <c r="C24" s="31" t="n">
+        <v>5.93</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1512,7 +1674,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1562,7 +1724,7 @@
           <t>Q design</t>
         </is>
       </c>
-      <c r="B4" s="17" t="n">
+      <c r="B4" s="32" t="n">
         <v>3.598</v>
       </c>
       <c r="C4" s="16" t="inlineStr">
@@ -1582,7 +1744,7 @@
           <t>S</t>
         </is>
       </c>
-      <c r="B5" s="17" t="n">
+      <c r="B5" s="32" t="n">
         <v>0.0173</v>
       </c>
       <c r="C5" s="16" t="inlineStr">
@@ -1602,7 +1764,7 @@
           <t>n Manning</t>
         </is>
       </c>
-      <c r="B6" s="17" t="n">
+      <c r="B6" s="32" t="n">
         <v>0.03</v>
       </c>
       <c r="C6" s="16" t="inlineStr">
@@ -1622,7 +1784,7 @@
           <t>z talus</t>
         </is>
       </c>
-      <c r="B7" s="17" t="n">
+      <c r="B7" s="32" t="n">
         <v>2</v>
       </c>
       <c r="C7" s="16" t="inlineStr">
@@ -1648,7 +1810,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1710,7 +1872,7 @@
           <t>Q</t>
         </is>
       </c>
-      <c r="C5" s="17" t="n">
+      <c r="C5" s="32" t="n">
         <v>3.598</v>
       </c>
       <c r="D5" s="16" t="inlineStr">
@@ -1730,7 +1892,7 @@
           <t>S</t>
         </is>
       </c>
-      <c r="C6" s="17" t="n">
+      <c r="C6" s="32" t="n">
         <v>0.0173</v>
       </c>
       <c r="D6" s="16" t="inlineStr">
@@ -1750,7 +1912,7 @@
           <t>n</t>
         </is>
       </c>
-      <c r="C7" s="17" t="n">
+      <c r="C7" s="32" t="n">
         <v>0.03</v>
       </c>
       <c r="D7" s="16" t="inlineStr">
@@ -1770,7 +1932,7 @@
           <t>z</t>
         </is>
       </c>
-      <c r="C8" s="17" t="n">
+      <c r="C8" s="32" t="n">
         <v>2</v>
       </c>
       <c r="D8" s="16" t="inlineStr">
@@ -1810,7 +1972,7 @@
           <t>x</t>
         </is>
       </c>
-      <c r="C10" s="19" t="n">
+      <c r="C10" s="33" t="n">
         <v>3.534</v>
       </c>
       <c r="D10" s="16" t="inlineStr">
@@ -1859,7 +2021,7 @@
           <t>A = (x + z*y)*y</t>
         </is>
       </c>
-      <c r="C14" s="13">
+      <c r="C14" s="27">
         <f>($C$10+$C$8*$C$9)*$C$9</f>
         <v/>
       </c>
@@ -1880,7 +2042,7 @@
           <t>P = x + 2*y*SQRT(1+z^2)</t>
         </is>
       </c>
-      <c r="C15" s="13">
+      <c r="C15" s="27">
         <f>$C$10+2*$C$9*SQRT(1+$C$8^2)</f>
         <v/>
       </c>
@@ -1901,7 +2063,7 @@
           <t>R = A/P</t>
         </is>
       </c>
-      <c r="C16" s="13">
+      <c r="C16" s="27">
         <f>C14/C15</f>
         <v/>
       </c>
@@ -1922,7 +2084,7 @@
           <t>Tw = x + 2*z*y</t>
         </is>
       </c>
-      <c r="C17" s="13">
+      <c r="C17" s="27">
         <f>$C$10+2*$C$8*$C$9</f>
         <v/>
       </c>
@@ -1943,7 +2105,7 @@
           <t>Q = (1/n)*A*R^(2/3)*SQRT(S)</t>
         </is>
       </c>
-      <c r="C18" s="13">
+      <c r="C18" s="27">
         <f>(1/$C$7)*C14*C16^(2/3)*SQRT($C$6)</f>
         <v/>
       </c>
@@ -1964,7 +2126,7 @@
           <t>V = Q/A</t>
         </is>
       </c>
-      <c r="C19" s="13">
+      <c r="C19" s="27">
         <f>C18/C14</f>
         <v/>
       </c>
@@ -1985,7 +2147,7 @@
           <t>Q ≈ Q design ?</t>
         </is>
       </c>
-      <c r="C20" s="13">
+      <c r="C20" s="27">
         <f>C18-$C$5</f>
         <v/>
       </c>
@@ -2024,7 +2186,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2091,19 +2253,19 @@
       <c r="A5" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="B5" s="13" t="n">
+      <c r="B5" s="27" t="n">
         <v>9.914999999999999</v>
       </c>
-      <c r="C5" s="13" t="n">
+      <c r="C5" s="27" t="n">
         <v>11.917</v>
       </c>
-      <c r="D5" s="13" t="n">
+      <c r="D5" s="27" t="n">
         <v>13.918</v>
       </c>
-      <c r="E5" s="13" t="n">
+      <c r="E5" s="27" t="n">
         <v>12.717</v>
       </c>
-      <c r="F5" s="13" t="n">
+      <c r="F5" s="27" t="n">
         <v>1.461</v>
       </c>
     </row>
@@ -2111,19 +2273,19 @@
       <c r="A6" s="18" t="n">
         <v>0.25</v>
       </c>
-      <c r="B6" s="13" t="n">
+      <c r="B6" s="27" t="n">
         <v>6.778</v>
       </c>
-      <c r="C6" s="13" t="n">
+      <c r="C6" s="27" t="n">
         <v>8.161</v>
       </c>
-      <c r="D6" s="13" t="n">
+      <c r="D6" s="27" t="n">
         <v>9.542</v>
       </c>
-      <c r="E6" s="13" t="n">
+      <c r="E6" s="27" t="n">
         <v>9.161</v>
       </c>
-      <c r="F6" s="13" t="n">
+      <c r="F6" s="27" t="n">
         <v>1.662</v>
       </c>
     </row>
@@ -2131,19 +2293,19 @@
       <c r="A7" s="18" t="n">
         <v>0.3</v>
       </c>
-      <c r="B7" s="13" t="n">
+      <c r="B7" s="27" t="n">
         <v>4.932</v>
       </c>
-      <c r="C7" s="13" t="n">
+      <c r="C7" s="27" t="n">
         <v>5.956</v>
       </c>
-      <c r="D7" s="13" t="n">
+      <c r="D7" s="27" t="n">
         <v>6.979</v>
       </c>
-      <c r="E7" s="13" t="n">
+      <c r="E7" s="27" t="n">
         <v>7.156</v>
       </c>
-      <c r="F7" s="13" t="n">
+      <c r="F7" s="27" t="n">
         <v>1.829</v>
       </c>
     </row>
@@ -2151,19 +2313,19 @@
       <c r="A8" s="18" t="n">
         <v>0.35</v>
       </c>
-      <c r="B8" s="13" t="n">
+      <c r="B8" s="27" t="n">
         <v>3.731</v>
       </c>
-      <c r="C8" s="13" t="n">
+      <c r="C8" s="27" t="n">
         <v>4.529</v>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="27" t="n">
         <v>5.324</v>
       </c>
-      <c r="E8" s="13" t="n">
+      <c r="E8" s="27" t="n">
         <v>5.929</v>
       </c>
-      <c r="F8" s="13" t="n">
+      <c r="F8" s="27" t="n">
         <v>1.966</v>
       </c>
     </row>
@@ -2171,19 +2333,19 @@
       <c r="A9" s="18" t="n">
         <v>0.4</v>
       </c>
-      <c r="B9" s="13" t="n">
+      <c r="B9" s="27" t="n">
         <v>2.889</v>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="27" t="n">
         <v>3.534</v>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" s="27" t="n">
         <v>4.175</v>
       </c>
-      <c r="E9" s="13" t="n">
+      <c r="E9" s="27" t="n">
         <v>5.134</v>
       </c>
-      <c r="F9" s="13" t="n">
+      <c r="F9" s="27" t="n">
         <v>2.075</v>
       </c>
     </row>
@@ -2191,19 +2353,19 @@
       <c r="A10" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="B10" s="13" t="n">
+      <c r="B10" s="27" t="n">
         <v>1.776</v>
       </c>
-      <c r="C10" s="13" t="n">
+      <c r="C10" s="27" t="n">
         <v>2.233</v>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" s="27" t="n">
         <v>2.686</v>
       </c>
-      <c r="E10" s="13" t="n">
+      <c r="E10" s="27" t="n">
         <v>4.233</v>
       </c>
-      <c r="F10" s="13" t="n">
+      <c r="F10" s="27" t="n">
         <v>2.226</v>
       </c>
     </row>
@@ -2211,19 +2373,19 @@
       <c r="A11" s="18" t="n">
         <v>0.6</v>
       </c>
-      <c r="B11" s="13" t="n">
+      <c r="B11" s="27" t="n">
         <v>1.047</v>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C11" s="27" t="n">
         <v>1.398</v>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="27" t="n">
         <v>1.744</v>
       </c>
-      <c r="E11" s="13" t="n">
+      <c r="E11" s="27" t="n">
         <v>3.798</v>
       </c>
-      <c r="F11" s="13" t="n">
+      <c r="F11" s="27" t="n">
         <v>2.308</v>
       </c>
     </row>
@@ -2231,19 +2393,19 @@
       <c r="A12" s="18" t="n">
         <v>0.7</v>
       </c>
-      <c r="B12" s="13" t="n">
+      <c r="B12" s="27" t="n">
         <v>0.506</v>
       </c>
-      <c r="C12" s="13" t="n">
+      <c r="C12" s="27" t="n">
         <v>0.792</v>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" s="27" t="n">
         <v>1.071</v>
       </c>
-      <c r="E12" s="13" t="n">
+      <c r="E12" s="27" t="n">
         <v>3.592</v>
       </c>
-      <c r="F12" s="13" t="n">
+      <c r="F12" s="27" t="n">
         <v>2.345</v>
       </c>
     </row>
@@ -2251,19 +2413,19 @@
       <c r="A13" s="18" t="n">
         <v>0.76</v>
       </c>
-      <c r="B13" s="13" t="n">
+      <c r="B13" s="27" t="n">
         <v>0.235</v>
       </c>
-      <c r="C13" s="13" t="n">
+      <c r="C13" s="27" t="n">
         <v>0.492</v>
       </c>
-      <c r="D13" s="13" t="n">
+      <c r="D13" s="27" t="n">
         <v>0.743</v>
       </c>
-      <c r="E13" s="13" t="n">
+      <c r="E13" s="27" t="n">
         <v>3.532</v>
       </c>
-      <c r="F13" s="13" t="n">
+      <c r="F13" s="27" t="n">
         <v>2.353</v>
       </c>
     </row>
@@ -2271,19 +2433,19 @@
       <c r="A14" s="18" t="n">
         <v>0.8</v>
       </c>
-      <c r="B14" s="13" t="n">
+      <c r="B14" s="27" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="C14" s="13" t="n">
+      <c r="C14" s="27" t="n">
         <v>0.311</v>
       </c>
-      <c r="D14" s="13" t="n">
+      <c r="D14" s="27" t="n">
         <v>0.546</v>
       </c>
-      <c r="E14" s="13" t="n">
+      <c r="E14" s="27" t="n">
         <v>3.511</v>
       </c>
-      <c r="F14" s="13" t="n">
+      <c r="F14" s="27" t="n">
         <v>2.353</v>
       </c>
     </row>
@@ -2291,19 +2453,19 @@
       <c r="A15" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="B15" s="13" t="n">
+      <c r="B15" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="C15" s="13" t="n">
+      <c r="C15" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="13" t="n">
+      <c r="D15" s="27" t="n">
         <v>0.11</v>
       </c>
-      <c r="E15" s="13" t="n">
+      <c r="E15" s="27" t="n">
         <v>3.6</v>
       </c>
-      <c r="F15" s="13" t="n">
+      <c r="F15" s="27" t="n">
         <v>2.221</v>
       </c>
     </row>
@@ -2311,19 +2473,19 @@
       <c r="A16" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="B16" s="13" t="n">
+      <c r="B16" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="C16" s="13" t="n">
+      <c r="C16" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="D16" s="13" t="n">
+      <c r="D16" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="E16" s="13" t="n">
+      <c r="E16" s="27" t="n">
         <v>4</v>
       </c>
-      <c r="F16" s="13" t="n">
+      <c r="F16" s="27" t="n">
         <v>1.799</v>
       </c>
     </row>
@@ -2339,7 +2501,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2432,7 +2594,7 @@
           <t>Q design (cible)</t>
         </is>
       </c>
-      <c r="B12" s="20">
+      <c r="B12" s="34">
         <f>Inputs!B4</f>
         <v/>
       </c>
@@ -2448,7 +2610,7 @@
           <t>S</t>
         </is>
       </c>
-      <c r="B13" s="20">
+      <c r="B13" s="34">
         <f>Inputs!B5</f>
         <v/>
       </c>
@@ -2464,7 +2626,7 @@
           <t>n</t>
         </is>
       </c>
-      <c r="B14" s="20">
+      <c r="B14" s="34">
         <f>Inputs!B6</f>
         <v/>
       </c>
@@ -2480,7 +2642,7 @@
           <t>z</t>
         </is>
       </c>
-      <c r="B15" s="20">
+      <c r="B15" s="34">
         <f>Inputs!B7</f>
         <v/>
       </c>
@@ -2496,7 +2658,7 @@
           <t>y (choix)</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n">
+      <c r="B16" s="32" t="n">
         <v>0.4</v>
       </c>
       <c r="C16" s="16" t="inlineStr">
@@ -2511,7 +2673,7 @@
           <t>x (essai / résultat)</t>
         </is>
       </c>
-      <c r="B17" s="17" t="n">
+      <c r="B17" s="32" t="n">
         <v>3.534</v>
       </c>
       <c r="C17" s="16" t="inlineStr">
@@ -2526,7 +2688,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="B19" s="13">
+      <c r="B19" s="27">
         <f>($B$17+$B$15*$B$16)*$B$16</f>
         <v/>
       </c>
@@ -2537,7 +2699,7 @@
           <t>P</t>
         </is>
       </c>
-      <c r="B20" s="13">
+      <c r="B20" s="27">
         <f>$B$17+2*$B$16*SQRT(1+$B$15^2)</f>
         <v/>
       </c>
@@ -2548,7 +2710,7 @@
           <t>R</t>
         </is>
       </c>
-      <c r="B21" s="13">
+      <c r="B21" s="27">
         <f>B19/B20</f>
         <v/>
       </c>
@@ -2559,7 +2721,7 @@
           <t>Tw</t>
         </is>
       </c>
-      <c r="B22" s="13">
+      <c r="B22" s="27">
         <f>$B$17+2*$B$15*$B$16</f>
         <v/>
       </c>
@@ -2570,7 +2732,7 @@
           <t>Q calc</t>
         </is>
       </c>
-      <c r="B23" s="22">
+      <c r="B23" s="35">
         <f>(1/$B$14)*B19*B21^(2/3)*SQRT($B$13)</f>
         <v/>
       </c>
@@ -2586,7 +2748,7 @@
           <t>V</t>
         </is>
       </c>
-      <c r="B24" s="13">
+      <c r="B24" s="27">
         <f>B23/B19</f>
         <v/>
       </c>

</xml_diff>